<commit_message>
MAJ Tableau des compétences
</commit_message>
<xml_diff>
--- a/assets/data/Tableau de compétences.xlsx
+++ b/assets/data/Tableau de compétences.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vxlle\OneDrive\Documents\Développement WEB\Projets\Portfolio PETIT Valentin restyle\Website\assets\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99896C07-0C10-492A-B9AD-74A0FFBE5053}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84BC09C5-FB1C-4F79-B70C-4B748CAA2740}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="36">
   <si>
     <t>Gérer le patrimoine informatique</t>
   </si>
@@ -131,7 +131,25 @@
     <t>Projet 1 - GereTonFrig</t>
   </si>
   <si>
-    <t>Projet 2 - Valen Facture</t>
+    <t>Projet 2 - Valen Budget</t>
+  </si>
+  <si>
+    <t>Création d'API</t>
+  </si>
+  <si>
+    <t>Projet apprentissage Marmiton</t>
+  </si>
+  <si>
+    <t>SAP : Gestion des rôles et accès</t>
+  </si>
+  <si>
+    <t>EDI : Développement continu et nouveaux partenaires</t>
+  </si>
+  <si>
+    <t>SAP : Migration vers ECC6 EHP8</t>
+  </si>
+  <si>
+    <t>WINDOWS + LINUX : Scripts et tâches planifiées</t>
   </si>
 </sst>
 </file>
@@ -141,7 +159,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$€-1]_-;\-* #,##0.00\ [$€-1]_-;_-* &quot;-&quot;??\ [$€-1]_-"/>
   </numFmts>
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -203,6 +221,12 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FFFF0000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -609,7 +633,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -671,15 +695,48 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -713,37 +770,16 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1065,56 +1101,56 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:43" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="24" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="23"/>
-      <c r="C1" s="23"/>
-      <c r="D1" s="23"/>
-      <c r="E1" s="23"/>
-      <c r="F1" s="23"/>
-      <c r="G1" s="23" t="s">
+      <c r="B1" s="24"/>
+      <c r="C1" s="24"/>
+      <c r="D1" s="24"/>
+      <c r="E1" s="24"/>
+      <c r="F1" s="24"/>
+      <c r="G1" s="24" t="s">
         <v>21</v>
       </c>
-      <c r="H1" s="23"/>
+      <c r="H1" s="24"/>
     </row>
     <row r="2" spans="1:43" ht="41.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="23" t="s">
+      <c r="A2" s="24" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="23"/>
-      <c r="C2" s="23"/>
-      <c r="D2" s="23"/>
-      <c r="E2" s="23"/>
-      <c r="F2" s="23"/>
-      <c r="G2" s="23"/>
-      <c r="H2" s="23"/>
+      <c r="B2" s="24"/>
+      <c r="C2" s="24"/>
+      <c r="D2" s="24"/>
+      <c r="E2" s="24"/>
+      <c r="F2" s="24"/>
+      <c r="G2" s="24"/>
+      <c r="H2" s="24"/>
     </row>
     <row r="3" spans="1:43" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="35" t="s">
+      <c r="A3" s="25" t="s">
         <v>24</v>
       </c>
-      <c r="B3" s="36"/>
-      <c r="C3" s="36"/>
-      <c r="D3" s="36"/>
-      <c r="E3" s="37"/>
-      <c r="F3" s="41" t="s">
+      <c r="B3" s="26"/>
+      <c r="C3" s="26"/>
+      <c r="D3" s="26"/>
+      <c r="E3" s="27"/>
+      <c r="F3" s="31" t="s">
         <v>22</v>
       </c>
-      <c r="G3" s="36"/>
-      <c r="H3" s="42"/>
+      <c r="G3" s="26"/>
+      <c r="H3" s="32"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
     </row>
     <row r="4" spans="1:43" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="38" t="s">
+      <c r="A4" s="28" t="s">
         <v>25</v>
       </c>
-      <c r="B4" s="39"/>
-      <c r="C4" s="39"/>
-      <c r="D4" s="39"/>
-      <c r="E4" s="40"/>
+      <c r="B4" s="29"/>
+      <c r="C4" s="29"/>
+      <c r="D4" s="29"/>
+      <c r="E4" s="30"/>
       <c r="F4" s="14" t="s">
         <v>8</v>
       </c>
@@ -1126,22 +1162,22 @@
       </c>
     </row>
     <row r="5" spans="1:43" ht="39.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="32" t="s">
+      <c r="A5" s="43" t="s">
         <v>26</v>
       </c>
-      <c r="B5" s="33"/>
-      <c r="C5" s="33"/>
-      <c r="D5" s="33"/>
-      <c r="E5" s="33"/>
-      <c r="F5" s="33"/>
-      <c r="G5" s="33"/>
-      <c r="H5" s="34"/>
+      <c r="B5" s="44"/>
+      <c r="C5" s="44"/>
+      <c r="D5" s="44"/>
+      <c r="E5" s="44"/>
+      <c r="F5" s="44"/>
+      <c r="G5" s="44"/>
+      <c r="H5" s="45"/>
     </row>
     <row r="6" spans="1:43" ht="90" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="21" t="s">
+      <c r="A6" s="33" t="s">
         <v>17</v>
       </c>
-      <c r="B6" s="30" t="s">
+      <c r="B6" s="41" t="s">
         <v>18</v>
       </c>
       <c r="C6" s="6" t="s">
@@ -1164,8 +1200,8 @@
       </c>
     </row>
     <row r="7" spans="1:43" s="2" customFormat="1" ht="324.89999999999998" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="22"/>
-      <c r="B7" s="31"/>
+      <c r="A7" s="34"/>
+      <c r="B7" s="42"/>
       <c r="C7" s="8" t="s">
         <v>9</v>
       </c>
@@ -1221,16 +1257,16 @@
       <c r="AQ7"/>
     </row>
     <row r="8" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
-      <c r="A8" s="24" t="s">
+      <c r="A8" s="35" t="s">
         <v>16</v>
       </c>
-      <c r="B8" s="25"/>
-      <c r="C8" s="25"/>
-      <c r="D8" s="25"/>
-      <c r="E8" s="25"/>
-      <c r="F8" s="25"/>
-      <c r="G8" s="25"/>
-      <c r="H8" s="26"/>
+      <c r="B8" s="36"/>
+      <c r="C8" s="36"/>
+      <c r="D8" s="36"/>
+      <c r="E8" s="36"/>
+      <c r="F8" s="36"/>
+      <c r="G8" s="36"/>
+      <c r="H8" s="37"/>
       <c r="I8"/>
       <c r="J8"/>
       <c r="K8"/>
@@ -1272,12 +1308,12 @@
         <v>27</v>
       </c>
       <c r="B9" s="10"/>
-      <c r="C9" s="45"/>
-      <c r="D9" s="44"/>
-      <c r="E9" s="44"/>
+      <c r="C9" s="23"/>
+      <c r="D9" s="22"/>
+      <c r="E9" s="22"/>
       <c r="F9" s="16"/>
       <c r="G9" s="16"/>
-      <c r="H9" s="43"/>
+      <c r="H9" s="21"/>
       <c r="I9"/>
       <c r="J9"/>
       <c r="K9"/>
@@ -1319,12 +1355,12 @@
         <v>28</v>
       </c>
       <c r="B10" s="10"/>
-      <c r="C10" s="44"/>
-      <c r="D10" s="44"/>
-      <c r="E10" s="44"/>
-      <c r="F10" s="44"/>
-      <c r="G10" s="44"/>
-      <c r="H10" s="43"/>
+      <c r="C10" s="22"/>
+      <c r="D10" s="22"/>
+      <c r="E10" s="22"/>
+      <c r="F10" s="22"/>
+      <c r="G10" s="22"/>
+      <c r="H10" s="21"/>
       <c r="I10"/>
       <c r="J10"/>
       <c r="K10"/>
@@ -1366,12 +1402,12 @@
         <v>29</v>
       </c>
       <c r="B11" s="10"/>
-      <c r="C11" s="44"/>
-      <c r="D11" s="44"/>
-      <c r="E11" s="44"/>
-      <c r="F11" s="44"/>
-      <c r="G11" s="44"/>
-      <c r="H11" s="43"/>
+      <c r="C11" s="22"/>
+      <c r="D11" s="22"/>
+      <c r="E11" s="22"/>
+      <c r="F11" s="22"/>
+      <c r="G11" s="22"/>
+      <c r="H11" s="21"/>
       <c r="I11"/>
       <c r="J11"/>
       <c r="K11"/>
@@ -1409,14 +1445,16 @@
       <c r="AQ11"/>
     </row>
     <row r="12" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="11"/>
+      <c r="A12" s="11" t="s">
+        <v>30</v>
+      </c>
       <c r="B12" s="10"/>
       <c r="C12" s="16"/>
       <c r="D12" s="16"/>
       <c r="E12" s="16"/>
-      <c r="F12" s="16"/>
+      <c r="F12" s="22"/>
       <c r="G12" s="16"/>
-      <c r="H12" s="17"/>
+      <c r="H12" s="21"/>
       <c r="I12"/>
       <c r="J12"/>
       <c r="K12"/>
@@ -1454,14 +1492,16 @@
       <c r="AQ12"/>
     </row>
     <row r="13" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="11"/>
+      <c r="A13" s="11" t="s">
+        <v>31</v>
+      </c>
       <c r="B13" s="10"/>
       <c r="C13" s="16"/>
       <c r="D13" s="16"/>
       <c r="E13" s="16"/>
-      <c r="F13" s="16"/>
+      <c r="F13" s="22"/>
       <c r="G13" s="16"/>
-      <c r="H13" s="17"/>
+      <c r="H13" s="21"/>
       <c r="I13"/>
       <c r="J13"/>
       <c r="K13"/>
@@ -1724,16 +1764,16 @@
       <c r="AQ18"/>
     </row>
     <row r="19" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
-      <c r="A19" s="27" t="s">
+      <c r="A19" s="38" t="s">
         <v>19</v>
       </c>
-      <c r="B19" s="28"/>
-      <c r="C19" s="28"/>
-      <c r="D19" s="28"/>
-      <c r="E19" s="28"/>
-      <c r="F19" s="28"/>
-      <c r="G19" s="28"/>
-      <c r="H19" s="29"/>
+      <c r="B19" s="39"/>
+      <c r="C19" s="39"/>
+      <c r="D19" s="39"/>
+      <c r="E19" s="39"/>
+      <c r="F19" s="39"/>
+      <c r="G19" s="39"/>
+      <c r="H19" s="40"/>
       <c r="I19"/>
       <c r="J19"/>
       <c r="K19"/>
@@ -1771,14 +1811,16 @@
       <c r="AQ19"/>
     </row>
     <row r="20" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="11"/>
-      <c r="B20" s="10"/>
-      <c r="C20" s="16"/>
-      <c r="D20" s="16"/>
+      <c r="A20" t="s">
+        <v>32</v>
+      </c>
+      <c r="B20" s="46"/>
+      <c r="C20" s="22"/>
+      <c r="D20" s="22"/>
       <c r="E20" s="16"/>
       <c r="F20" s="16"/>
-      <c r="G20" s="16"/>
-      <c r="H20" s="17"/>
+      <c r="G20" s="49"/>
+      <c r="H20" s="48"/>
       <c r="I20"/>
       <c r="J20"/>
       <c r="K20"/>
@@ -1816,14 +1858,16 @@
       <c r="AQ20"/>
     </row>
     <row r="21" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="11"/>
+      <c r="A21" t="s">
+        <v>33</v>
+      </c>
       <c r="B21" s="10"/>
-      <c r="C21" s="16"/>
-      <c r="D21" s="16"/>
-      <c r="E21" s="16"/>
-      <c r="F21" s="16"/>
-      <c r="G21" s="16"/>
-      <c r="H21" s="17"/>
+      <c r="C21" s="47"/>
+      <c r="D21" s="22"/>
+      <c r="E21" s="22"/>
+      <c r="F21" s="47"/>
+      <c r="G21" s="22"/>
+      <c r="H21" s="21"/>
       <c r="I21"/>
       <c r="J21"/>
       <c r="K21"/>
@@ -1861,7 +1905,9 @@
       <c r="AQ21"/>
     </row>
     <row r="22" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="11"/>
+      <c r="A22" t="s">
+        <v>35</v>
+      </c>
       <c r="B22" s="10"/>
       <c r="C22" s="16"/>
       <c r="D22" s="16"/>
@@ -2086,16 +2132,16 @@
       <c r="AQ26"/>
     </row>
     <row r="27" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
-      <c r="A27" s="27" t="s">
+      <c r="A27" s="38" t="s">
         <v>20</v>
       </c>
-      <c r="B27" s="28"/>
-      <c r="C27" s="28"/>
-      <c r="D27" s="28"/>
-      <c r="E27" s="28"/>
-      <c r="F27" s="28"/>
-      <c r="G27" s="28"/>
-      <c r="H27" s="29"/>
+      <c r="B27" s="39"/>
+      <c r="C27" s="39"/>
+      <c r="D27" s="39"/>
+      <c r="E27" s="39"/>
+      <c r="F27" s="39"/>
+      <c r="G27" s="39"/>
+      <c r="H27" s="40"/>
       <c r="I27"/>
       <c r="J27"/>
       <c r="K27"/>
@@ -2133,14 +2179,16 @@
       <c r="AQ27"/>
     </row>
     <row r="28" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="11"/>
-      <c r="B28" s="10"/>
-      <c r="C28" s="16"/>
-      <c r="D28" s="16"/>
+      <c r="A28" t="s">
+        <v>32</v>
+      </c>
+      <c r="B28" s="46"/>
+      <c r="C28" s="22"/>
+      <c r="D28" s="22"/>
       <c r="E28" s="16"/>
       <c r="F28" s="16"/>
-      <c r="G28" s="16"/>
-      <c r="H28" s="17"/>
+      <c r="G28" s="22"/>
+      <c r="H28" s="48"/>
       <c r="I28"/>
       <c r="J28"/>
       <c r="K28"/>
@@ -2178,14 +2226,16 @@
       <c r="AQ28"/>
     </row>
     <row r="29" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="11"/>
+      <c r="A29" t="s">
+        <v>33</v>
+      </c>
       <c r="B29" s="10"/>
-      <c r="C29" s="16"/>
-      <c r="D29" s="16"/>
-      <c r="E29" s="16"/>
-      <c r="F29" s="16"/>
-      <c r="G29" s="16"/>
-      <c r="H29" s="17"/>
+      <c r="C29" s="47"/>
+      <c r="D29" s="22"/>
+      <c r="E29" s="22"/>
+      <c r="F29" s="47"/>
+      <c r="G29" s="22"/>
+      <c r="H29" s="21"/>
       <c r="I29"/>
       <c r="J29"/>
       <c r="K29"/>
@@ -2223,14 +2273,16 @@
       <c r="AQ29"/>
     </row>
     <row r="30" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="11"/>
+      <c r="A30" t="s">
+        <v>34</v>
+      </c>
       <c r="B30" s="10"/>
-      <c r="C30" s="16"/>
+      <c r="C30" s="22"/>
       <c r="D30" s="16"/>
       <c r="E30" s="16"/>
       <c r="F30" s="16"/>
-      <c r="G30" s="16"/>
-      <c r="H30" s="17"/>
+      <c r="G30" s="22"/>
+      <c r="H30" s="21"/>
       <c r="I30"/>
       <c r="J30"/>
       <c r="K30"/>
@@ -2268,12 +2320,14 @@
       <c r="AQ30"/>
     </row>
     <row r="31" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="11"/>
+      <c r="A31" t="s">
+        <v>35</v>
+      </c>
       <c r="B31" s="10"/>
-      <c r="C31" s="16"/>
-      <c r="D31" s="16"/>
+      <c r="C31" s="22"/>
+      <c r="D31" s="22"/>
       <c r="E31" s="16"/>
-      <c r="F31" s="16"/>
+      <c r="F31" s="22"/>
       <c r="G31" s="16"/>
       <c r="H31" s="17"/>
       <c r="I31"/>
@@ -2540,11 +2594,6 @@
     <row r="81" customFormat="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="G1:H1"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A3:E3"/>
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="F3:H3"/>
     <mergeCell ref="A6:A7"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A8:H8"/>
@@ -2552,6 +2601,11 @@
     <mergeCell ref="A27:H27"/>
     <mergeCell ref="B6:B7"/>
     <mergeCell ref="A5:H5"/>
+    <mergeCell ref="G1:H1"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="F3:H3"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <printOptions horizontalCentered="1" verticalCentered="1"/>

</xml_diff>